<commit_message>
chore: update project and add allure screenshot script
</commit_message>
<xml_diff>
--- a/data/cases/login_cases.xlsx
+++ b/data/cases/login_cases.xlsx
@@ -588,7 +588,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>用户名首尾空格</t>
+          <t>用户名首尾空格自动去除后登录</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -603,7 +603,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>success</t>
         </is>
       </c>
       <c r="E8" t="b">

</xml_diff>